<commit_message>
docs: record feature audit implementation receipt
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R713fafc213334888"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R10cbfd46b1734f21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R5064617c9934415f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rb2a019f91e4740e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rdd316f09a72e4bdb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Re211c15ac10340e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R4b60ca0280694a81"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R588216baf022468c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -728,7 +728,9 @@
       <x:c r="R3" s="14" t="str">
         <x:v>index.html</x:v>
       </x:c>
-      <x:c r="S3" s="14" t="str"/>
+      <x:c r="S3" s="14" t="str">
+        <x:v>4883949</x:v>
+      </x:c>
       <x:c r="T3" s="14" t="str">
         <x:v>Open / at 390x844; activate Menu; inspect class and aria-expanded; verify links; measure document overflow.</x:v>
       </x:c>
@@ -1518,7 +1520,9 @@
       <x:c r="R15" s="14" t="str">
         <x:v>cmd/server/demo_ui.go; cmd/server/demo_ui_test.go</x:v>
       </x:c>
-      <x:c r="S15" s="14" t="str"/>
+      <x:c r="S15" s="14" t="str">
+        <x:v>4883949</x:v>
+      </x:c>
       <x:c r="T15" s="14" t="str">
         <x:v>Enumerate CTA links and accessible names; validate local links; inspect visual priority and mobile wrapping.</x:v>
       </x:c>
@@ -1788,7 +1792,9 @@
       <x:c r="R19" s="14" t="str">
         <x:v>index.html</x:v>
       </x:c>
-      <x:c r="S19" s="14" t="str"/>
+      <x:c r="S19" s="14" t="str">
+        <x:v>4883949</x:v>
+      </x:c>
       <x:c r="T19" s="14" t="str">
         <x:v>Open /?tour=1 at 1920x1080; assert theater visible, Apple opening, one stage, no overflow.</x:v>
       </x:c>
@@ -2773,7 +2779,9 @@
       <x:c r="R34" s="14" t="str">
         <x:v>cmd/server/demo_ui.go; cmd/server/demo_ui_test.go</x:v>
       </x:c>
-      <x:c r="S34" s="14" t="str"/>
+      <x:c r="S34" s="14" t="str">
+        <x:v>4883949</x:v>
+      </x:c>
       <x:c r="T34" s="14" t="str">
         <x:v>Run cmd/server route tests; render root HTML locally; inspect required copy, graphics, links, and responsive layout.</x:v>
       </x:c>
@@ -2848,7 +2856,9 @@
       <x:c r="R35" s="14" t="str">
         <x:v>cmd/server/demo_ui.go; cmd/server/demo_ui_test.go</x:v>
       </x:c>
-      <x:c r="S35" s="14" t="str"/>
+      <x:c r="S35" s="14" t="str">
+        <x:v>4883949</x:v>
+      </x:c>
       <x:c r="T35" s="14" t="str">
         <x:v>Run route test; render /demo; verify copy, SVG architecture, actions, responsive behavior, and non-advice framing.</x:v>
       </x:c>
@@ -3508,7 +3518,9 @@
       <x:c r="R45" s="14" t="str">
         <x:v>cmd/server/demo_ui.go; cmd/server/demo_ui_test.go</x:v>
       </x:c>
-      <x:c r="S45" s="14" t="str"/>
+      <x:c r="S45" s="14" t="str">
+        <x:v>4883949</x:v>
+      </x:c>
       <x:c r="T45" s="14" t="str">
         <x:v>Run local server; test three routes at desktop/mobile; keyboard through controls; Lighthouse snapshot; reduced-motion inspection.</x:v>
       </x:c>
@@ -4391,7 +4403,7 @@
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
-        <x:v>0</x:v>
+        <x:v>6</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
feat: add top-level project description
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rdd316f09a72e4bdb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Re211c15ac10340e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R4b60ca0280694a81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R588216baf022468c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rbd12a5889ac54635"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rbd17b9a567444fda"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R00ac701a373a49ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R5180e81f825c4d95"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4255,18 +4255,87 @@
         <x:v>/goal implement the cutting edge UI rich with graphics and easy to understand</x:v>
       </x:c>
     </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="14" t="str">
+        <x:v>WEB-018</x:v>
+      </x:c>
+      <x:c r="B57" s="14" t="str">
+        <x:v>Top-level project description</x:v>
+      </x:c>
+      <x:c r="C57" s="14" t="str">
+        <x:v>Landing / Hero</x:v>
+      </x:c>
+      <x:c r="D57" s="14" t="str">
+        <x:v>index.html; tests/landing-page.mjs</x:v>
+      </x:c>
+      <x:c r="E57" s="14" t="str">
+        <x:v>/ first viewport</x:v>
+      </x:c>
+      <x:c r="F57" s="14" t="str">
+        <x:v>First-time visitor</x:v>
+      </x:c>
+      <x:c r="G57" s="14" t="str">
+        <x:v>As a first-time visitor, I want a plain-language project description at the top so that I immediately understand what DeltaSignal is, what evidence it uses, and who it serves.</x:v>
+      </x:c>
+      <x:c r="H57" s="14" t="str">
+        <x:v>A visible description above the Apple reference identifies DeltaSignal as a governed financial-evidence operating system that turns dated filings and market data into provenance-rich research packets for AI agents and human analysts.</x:v>
+      </x:c>
+      <x:c r="I57" s="14" t="str">
+        <x:v>The project description is visible above the Apple case, uses concise plain language, and remains readable on desktop and mobile.</x:v>
+      </x:c>
+      <x:c r="J57" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K57" s="14" t="str">
+        <x:v>Automated UI</x:v>
+      </x:c>
+      <x:c r="L57" s="14" t="str">
+        <x:v>Load /; inspect the first viewport; assert the four defining phrases; verify visibility; rerun desktop and mobile landing tests.</x:v>
+      </x:c>
+      <x:c r="M57" s="14" t="str">
+        <x:v>PASS — qa_evidence/logs/project-description-test.log</x:v>
+      </x:c>
+      <x:c r="N57" s="14" t="str"/>
+      <x:c r="O57" s="14" t="str"/>
+      <x:c r="P57" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q57" s="14" t="str"/>
+      <x:c r="R57" s="14" t="str">
+        <x:v>index.html; tests/landing-page.mjs; CHANGELOG.html</x:v>
+      </x:c>
+      <x:c r="S57" s="14" t="str"/>
+      <x:c r="T57" s="14" t="str">
+        <x:v>Run node tests/landing-page.mjs.</x:v>
+      </x:c>
+      <x:c r="U57" s="14" t="str">
+        <x:v>PASS — landing-page: PASS</x:v>
+      </x:c>
+      <x:c r="V57" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W57" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X57" s="14" t="str">
+        <x:v>Added after the completed 55-story audit as the next tracker-backed homepage enhancement.</x:v>
+      </x:c>
+      <x:c r="Y57" s="14" t="str">
+        <x:v>at the top add description of the project</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="J2:J56">
+    <x:dataValidation type="list" sqref="J2:J57">
       <x:formula1>"Not Reviewed,Story Drafted,Ready For Test,Failed Test,Fix In Progress,Fixed,Retest Failed,Verified,Blocked,Needs Product Decision"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="O2:O56">
+    <x:dataValidation type="list" sqref="O2:O57">
       <x:formula1>"Critical,High,Medium,Low,None"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K2:K56">
+    <x:dataValidation type="list" sqref="K2:K57">
       <x:formula1>"Code Review,Manual UI,Automated Test,Smoke Test,Regression Test,Accessibility Review,Responsive Review,Integration Test"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="V2:V56">
+    <x:dataValidation type="list" sqref="V2:V57">
       <x:formula1>"Not Reviewed,Story Drafted,Ready For Test,Failed Test,Fix In Progress,Fixed,Retest Failed,Verified,Blocked,Needs Product Decision"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4316,14 +4385,14 @@
         <x:v>Tracked Features</x:v>
       </x:c>
       <x:c r="B4" s="21" t="n">
-        <x:f>COUNTA('Tracker'!$A$2:$A$56)</x:f>
-        <x:v>55</x:v>
+        <x:f>COUNTA('Tracker'!$A$2:$A$57)</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="E4" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$56,"Critical",'Tracker'!$V$2:$V$56,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"Critical",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4332,14 +4401,14 @@
         <x:v>Current Verified</x:v>
       </x:c>
       <x:c r="B5" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$56,"Verified")</x:f>
-        <x:v>49</x:v>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Verified")</x:f>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="E5" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$56,"High",'Tracker'!$V$2:$V$56,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"High",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4348,14 +4417,14 @@
         <x:v>Failed Test</x:v>
       </x:c>
       <x:c r="B6" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$56,"Failed Test")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Failed Test")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="21" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="E6" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$56,"Medium",'Tracker'!$V$2:$V$56,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"Medium",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4364,14 +4433,14 @@
         <x:v>Fix In Progress</x:v>
       </x:c>
       <x:c r="B7" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$56,"Fix In Progress")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Fix In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="E7" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$56,"Low",'Tracker'!$V$2:$V$56,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"Low",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4380,14 +4449,14 @@
         <x:v>Fixed</x:v>
       </x:c>
       <x:c r="B8" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$56,"Fixed")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Fixed")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="21" t="str">
         <x:v>Needs Product Decision</x:v>
       </x:c>
       <x:c r="E8" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$W$2:$W$56,"Yes")</x:f>
+        <x:f>COUNTIF('Tracker'!$W$2:$W$57,"Yes")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4396,8 +4465,8 @@
         <x:v>Final Verified</x:v>
       </x:c>
       <x:c r="B9" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$V$2:$V$56,"Verified")</x:f>
-        <x:v>55</x:v>
+        <x:f>COUNTIF('Tracker'!$V$2:$V$57,"Verified")</x:f>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
@@ -4411,7 +4480,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$V$2:$V$56,"Blocked")</x:f>
+        <x:f>COUNTIF('Tracker'!$V$2:$V$57,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
docs: record project description receipt
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rbd12a5889ac54635"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rbd17b9a567444fda"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R00ac701a373a49ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R5180e81f825c4d95"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R14a908993e1c44ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4fcfa27517ea4284"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R9fa9c60e680941bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R7abd86a699d54af1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4304,7 +4304,9 @@
       <x:c r="R57" s="14" t="str">
         <x:v>index.html; tests/landing-page.mjs; CHANGELOG.html</x:v>
       </x:c>
-      <x:c r="S57" s="14" t="str"/>
+      <x:c r="S57" s="14" t="str">
+        <x:v>9530d6a</x:v>
+      </x:c>
       <x:c r="T57" s="14" t="str">
         <x:v>Run node tests/landing-page.mjs.</x:v>
       </x:c>
@@ -4472,7 +4474,7 @@
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
-        <x:v>6</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
feat: explain daily SEC-to-agent evidence flow
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R14a908993e1c44ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R4fcfa27517ea4284"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R9fa9c60e680941bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R7abd86a699d54af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R2daa79ac6aeb4e5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc613ed0f2b854dc0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R80d6342e77cb4f3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rb160deb246d14aa4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4326,18 +4326,89 @@
         <x:v>at the top add description of the project</x:v>
       </x:c>
     </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="14" t="str">
+        <x:v>WEB-019</x:v>
+      </x:c>
+      <x:c r="B58" s="14" t="str">
+        <x:v>Daily SEC-to-MCP-to-Google-agents explanation</x:v>
+      </x:c>
+      <x:c r="C58" s="14" t="str">
+        <x:v>Landing / Hero</x:v>
+      </x:c>
+      <x:c r="D58" s="14" t="str">
+        <x:v>index.html; tests/landing-page.mjs</x:v>
+      </x:c>
+      <x:c r="E58" s="14" t="str">
+        <x:v>/ first viewport</x:v>
+      </x:c>
+      <x:c r="F58" s="14" t="str">
+        <x:v>First-time visitor / prospective client</x:v>
+      </x:c>
+      <x:c r="G58" s="14" t="str">
+        <x:v>As a first-time visitor, I want to see how DeltaSignal turns daily SEC evidence into an MCP-accessible database and how Google agents use it for Apple, so that I understand the product before opening the demo.</x:v>
+      </x:c>
+      <x:c r="H58" s="14" t="str">
+        <x:v>The first viewport shows four ordered and visible stages: collect public SEC/EDGAR and CompanyFacts/XBRL evidence; normalize, validate, date, hash, and materialize it in a governed evidence database; deliver bounded provenance-rich envelopes through read-only DeltaSignal MCP tools; and route AAPL questions through a Cloud Run coordinator to four bounded Google Cloud specialists without allowing Gemini explanation to replace source evidence.</x:v>
+      </x:c>
+      <x:c r="I58" s="14" t="str">
+        <x:v>The homepage now presents the complete daily SEC → governed evidence database → DeltaSignal MCP → Apple × Google Cloud agents sequence above the Apple reference case on desktop and mobile.</x:v>
+      </x:c>
+      <x:c r="J58" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K58" s="14" t="str">
+        <x:v>Automated UI</x:v>
+      </x:c>
+      <x:c r="L58" s="14" t="str">
+        <x:v>Load / on desktop and mobile; assert the workflow is visible; assert exactly four stages and all required SEC, database, MCP, Cloud Run, specialist-agent, and evidence-boundary phrases; verify no mobile horizontal overflow.</x:v>
+      </x:c>
+      <x:c r="M58" s="14" t="str">
+        <x:v>PASS — qa_evidence/logs/daily-sec-mcp-google-agents-test.log</x:v>
+      </x:c>
+      <x:c r="N58" s="14" t="str"/>
+      <x:c r="O58" s="14" t="str"/>
+      <x:c r="P58" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q58" s="14" t="str">
+        <x:v>Added a four-stage visual operating model and supporting automated assertions.</x:v>
+      </x:c>
+      <x:c r="R58" s="14" t="str">
+        <x:v>index.html; tests/landing-page.mjs; CHANGELOG.html</x:v>
+      </x:c>
+      <x:c r="S58" s="14" t="str"/>
+      <x:c r="T58" s="14" t="str">
+        <x:v>Run node tests/landing-page.mjs.</x:v>
+      </x:c>
+      <x:c r="U58" s="14" t="str">
+        <x:v>PASS — landing-page: PASS</x:v>
+      </x:c>
+      <x:c r="V58" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W58" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X58" s="14" t="str">
+        <x:v>Claims are bounded to the documented daily backend and Google Cloud AAPL client architecture; no claim that model-generated explanation replaces evidence.</x:v>
+      </x:c>
+      <x:c r="Y58" s="14" t="str">
+        <x:v>add description how deltasignal works every day collecting SEC information , creating db making it available to MCP, then describe how MCP is used in this example with Apple by creating ther agrents in google</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="J2:J57">
+    <x:dataValidation type="list" sqref="J2:J58">
       <x:formula1>"Not Reviewed,Story Drafted,Ready For Test,Failed Test,Fix In Progress,Fixed,Retest Failed,Verified,Blocked,Needs Product Decision"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="O2:O57">
+    <x:dataValidation type="list" sqref="O2:O58">
       <x:formula1>"Critical,High,Medium,Low,None"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K2:K57">
+    <x:dataValidation type="list" sqref="K2:K58">
       <x:formula1>"Code Review,Manual UI,Automated Test,Smoke Test,Regression Test,Accessibility Review,Responsive Review,Integration Test"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="V2:V57">
+    <x:dataValidation type="list" sqref="V2:V58">
       <x:formula1>"Not Reviewed,Story Drafted,Ready For Test,Failed Test,Fix In Progress,Fixed,Retest Failed,Verified,Blocked,Needs Product Decision"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4387,14 +4458,14 @@
         <x:v>Tracked Features</x:v>
       </x:c>
       <x:c r="B4" s="21" t="n">
-        <x:f>COUNTA('Tracker'!$A$2:$A$57)</x:f>
-        <x:v>56</x:v>
+        <x:f>COUNTA('Tracker'!$A$2:$A$58)</x:f>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="E4" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"Critical",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"Critical",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4403,14 +4474,14 @@
         <x:v>Current Verified</x:v>
       </x:c>
       <x:c r="B5" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Verified")</x:f>
-        <x:v>50</x:v>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Verified")</x:f>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="E5" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"High",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"High",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4419,14 +4490,14 @@
         <x:v>Failed Test</x:v>
       </x:c>
       <x:c r="B6" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Failed Test")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Failed Test")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="21" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="E6" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"Medium",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"Medium",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4435,14 +4506,14 @@
         <x:v>Fix In Progress</x:v>
       </x:c>
       <x:c r="B7" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Fix In Progress")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Fix In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="E7" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$57,"Low",'Tracker'!$V$2:$V$57,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"Low",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4451,14 +4522,14 @@
         <x:v>Fixed</x:v>
       </x:c>
       <x:c r="B8" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$57,"Fixed")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Fixed")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="21" t="str">
         <x:v>Needs Product Decision</x:v>
       </x:c>
       <x:c r="E8" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$W$2:$W$57,"Yes")</x:f>
+        <x:f>COUNTIF('Tracker'!$W$2:$W$58,"Yes")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4467,8 +4538,8 @@
         <x:v>Final Verified</x:v>
       </x:c>
       <x:c r="B9" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$V$2:$V$57,"Verified")</x:f>
-        <x:v>56</x:v>
+        <x:f>COUNTIF('Tracker'!$V$2:$V$58,"Verified")</x:f>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
@@ -4482,7 +4553,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$V$2:$V$57,"Blocked")</x:f>
+        <x:f>COUNTIF('Tracker'!$V$2:$V$58,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
docs: record SEC-to-agent feature receipt
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R2daa79ac6aeb4e5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Rc613ed0f2b854dc0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R80d6342e77cb4f3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Rb160deb246d14aa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R5d5bda9ee31f4c07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Raa55143ca0a64c37"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Re5030d816068444b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R159c910b77944c15"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4377,7 +4377,9 @@
       <x:c r="R58" s="14" t="str">
         <x:v>index.html; tests/landing-page.mjs; CHANGELOG.html</x:v>
       </x:c>
-      <x:c r="S58" s="14" t="str"/>
+      <x:c r="S58" s="14" t="str">
+        <x:v>220ee75</x:v>
+      </x:c>
       <x:c r="T58" s="14" t="str">
         <x:v>Run node tests/landing-page.mjs.</x:v>
       </x:c>
@@ -4545,7 +4547,7 @@
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
-        <x:v>7</x:v>
+        <x:v>8</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>

<commit_message>
feat: add agent-native evidence fabric infographic
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R5d5bda9ee31f4c07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="Raa55143ca0a64c37"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Re5030d816068444b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R159c910b77944c15"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R8ff37b255b97406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R67b9fe2daed141b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R914b87c9bcc24a41"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Re2ce38358d494387"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4399,18 +4399,89 @@
         <x:v>add description how deltasignal works every day collecting SEC information , creating db making it available to MCP, then describe how MCP is used in this example with Apple by creating ther agrents in google</x:v>
       </x:c>
     </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="14" t="str">
+        <x:v>WEB-020</x:v>
+      </x:c>
+      <x:c r="B59" s="14" t="str">
+        <x:v>Agent-native evidence-fabric infographic</x:v>
+      </x:c>
+      <x:c r="C59" s="14" t="str">
+        <x:v>Landing / Evidence Fabric</x:v>
+      </x:c>
+      <x:c r="D59" s="14" t="str">
+        <x:v>index.html; assets/deltasignal-agent-native-evidence-fabric.png; tests/landing-page.mjs</x:v>
+      </x:c>
+      <x:c r="E59" s="14" t="str">
+        <x:v>/ evidence-fabric section</x:v>
+      </x:c>
+      <x:c r="F59" s="14" t="str">
+        <x:v>First-time visitor / prospective client</x:v>
+      </x:c>
+      <x:c r="G59" s="14" t="str">
+        <x:v>As a visitor, I want one large infographic of the complete DeltaSignal workflow so that I can understand how SEC evidence becomes an Apple answer through MCP and Google Cloud agents.</x:v>
+      </x:c>
+      <x:c r="H59" s="14" t="str">
+        <x:v>A full-width, readable infographic appears after the trust strip and shows SEC/EDGAR and CompanyFacts/XBRL collection, governed materialization and storage, MCP delivery, and the bounded Apple Google Cloud agent runtime. The image has descriptive alternative text, a trust-boundary caption, responsive sizing, and no mobile overflow.</x:v>
+      </x:c>
+      <x:c r="I59" s="14" t="str">
+        <x:v>The supplied 2752×1536 infographic is presented in a responsive framed section with explanatory heading, accessible alternative text, and a caption preserving the missing-data and source-evidence boundary.</x:v>
+      </x:c>
+      <x:c r="J59" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="K59" s="14" t="str">
+        <x:v>Automated UI + visual inspection</x:v>
+      </x:c>
+      <x:c r="L59" s="14" t="str">
+        <x:v>Load /; scroll to the evidence-fabric section; assert exactly one image, expected source path, complete load, minimum 1200×800 natural dimensions, descriptive SEC EDGAR alt text, and no mobile overflow; visually inspect desktop rendering.</x:v>
+      </x:c>
+      <x:c r="M59" s="14" t="str">
+        <x:v>PASS — qa_evidence/logs/evidence-fabric-infographic-test.log</x:v>
+      </x:c>
+      <x:c r="N59" s="14" t="str"/>
+      <x:c r="O59" s="14" t="str"/>
+      <x:c r="P59" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="Q59" s="14" t="str">
+        <x:v>Added responsive infographic section, asset, caption, embedded visual-spec contract entry, and automated assertions.</x:v>
+      </x:c>
+      <x:c r="R59" s="14" t="str">
+        <x:v>index.html; assets/deltasignal-agent-native-evidence-fabric.png; tests/landing-page.mjs; CHANGELOG.html</x:v>
+      </x:c>
+      <x:c r="S59" s="14" t="str"/>
+      <x:c r="T59" s="14" t="str">
+        <x:v>Run node tests/landing-page.mjs and inspect desktop/mobile rendering.</x:v>
+      </x:c>
+      <x:c r="U59" s="14" t="str">
+        <x:v>PASS — landing-page: PASS</x:v>
+      </x:c>
+      <x:c r="V59" s="14" t="str">
+        <x:v>Verified</x:v>
+      </x:c>
+      <x:c r="W59" s="14" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="X59" s="14" t="str">
+        <x:v>The infographic is a supplied explanatory visual; the surrounding copy keeps evidence and model synthesis distinct.</x:v>
+      </x:c>
+      <x:c r="Y59" s="14" t="str">
+        <x:v>add the following infographic</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:dataValidations count="4">
-    <x:dataValidation type="list" sqref="J2:J58">
+    <x:dataValidation type="list" sqref="J2:J59">
       <x:formula1>"Not Reviewed,Story Drafted,Ready For Test,Failed Test,Fix In Progress,Fixed,Retest Failed,Verified,Blocked,Needs Product Decision"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="O2:O58">
+    <x:dataValidation type="list" sqref="O2:O59">
       <x:formula1>"Critical,High,Medium,Low,None"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="K2:K58">
+    <x:dataValidation type="list" sqref="K2:K59">
       <x:formula1>"Code Review,Manual UI,Automated Test,Smoke Test,Regression Test,Accessibility Review,Responsive Review,Integration Test"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="V2:V58">
+    <x:dataValidation type="list" sqref="V2:V59">
       <x:formula1>"Not Reviewed,Story Drafted,Ready For Test,Failed Test,Fix In Progress,Fixed,Retest Failed,Verified,Blocked,Needs Product Decision"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>
@@ -4460,14 +4531,14 @@
         <x:v>Tracked Features</x:v>
       </x:c>
       <x:c r="B4" s="21" t="n">
-        <x:f>COUNTA('Tracker'!$A$2:$A$58)</x:f>
-        <x:v>57</x:v>
+        <x:f>COUNTA('Tracker'!$A$2:$A$59)</x:f>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D4" s="21" t="str">
         <x:v>Critical</x:v>
       </x:c>
       <x:c r="E4" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"Critical",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$59,"Critical",'Tracker'!$V$2:$V$59,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4476,14 +4547,14 @@
         <x:v>Current Verified</x:v>
       </x:c>
       <x:c r="B5" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Verified")</x:f>
-        <x:v>51</x:v>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$59,"Verified")</x:f>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="D5" s="21" t="str">
         <x:v>High</x:v>
       </x:c>
       <x:c r="E5" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"High",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$59,"High",'Tracker'!$V$2:$V$59,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4492,14 +4563,14 @@
         <x:v>Failed Test</x:v>
       </x:c>
       <x:c r="B6" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Failed Test")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$59,"Failed Test")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D6" s="21" t="str">
         <x:v>Medium</x:v>
       </x:c>
       <x:c r="E6" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"Medium",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$59,"Medium",'Tracker'!$V$2:$V$59,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4508,14 +4579,14 @@
         <x:v>Fix In Progress</x:v>
       </x:c>
       <x:c r="B7" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Fix In Progress")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$59,"Fix In Progress")</x:f>
         <x:v>0</x:v>
       </x:c>
       <x:c r="D7" s="21" t="str">
         <x:v>Low</x:v>
       </x:c>
       <x:c r="E7" s="21" t="n">
-        <x:f>COUNTIFS('Tracker'!$O$2:$O$58,"Low",'Tracker'!$V$2:$V$58,"&lt;&gt;Verified")</x:f>
+        <x:f>COUNTIFS('Tracker'!$O$2:$O$59,"Low",'Tracker'!$V$2:$V$59,"&lt;&gt;Verified")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4524,14 +4595,14 @@
         <x:v>Fixed</x:v>
       </x:c>
       <x:c r="B8" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$J$2:$J$58,"Fixed")</x:f>
+        <x:f>COUNTIF('Tracker'!$J$2:$J$59,"Fixed")</x:f>
         <x:v>6</x:v>
       </x:c>
       <x:c r="D8" s="21" t="str">
         <x:v>Needs Product Decision</x:v>
       </x:c>
       <x:c r="E8" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$W$2:$W$58,"Yes")</x:f>
+        <x:f>COUNTIF('Tracker'!$W$2:$W$59,"Yes")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -4540,8 +4611,8 @@
         <x:v>Final Verified</x:v>
       </x:c>
       <x:c r="B9" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$V$2:$V$58,"Verified")</x:f>
-        <x:v>57</x:v>
+        <x:f>COUNTIF('Tracker'!$V$2:$V$59,"Verified")</x:f>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D9" s="21" t="str">
         <x:v>Rows With Commit Hash</x:v>
@@ -4555,7 +4626,7 @@
         <x:v>Blocked</x:v>
       </x:c>
       <x:c r="B10" s="21" t="n">
-        <x:f>COUNTIF('Tracker'!$V$2:$V$58,"Blocked")</x:f>
+        <x:f>COUNTIF('Tracker'!$V$2:$V$59,"Blocked")</x:f>
         <x:v>0</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
docs: record evidence fabric feature receipt
</commit_message>
<xml_diff>
--- a/feature_status_tracker.xlsx
+++ b/feature_status_tracker.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="R8ff37b255b97406c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R67b9fe2daed141b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="R914b87c9bcc24a41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="Re2ce38358d494387"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tracker" sheetId="1" r:id="Rd362b850e6a74b76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" r:id="R0b0fb128414545b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="3" r:id="Rcfb7fed3468244c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="4" r:id="R218346e9f0e04825"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4450,7 +4450,9 @@
       <x:c r="R59" s="14" t="str">
         <x:v>index.html; assets/deltasignal-agent-native-evidence-fabric.png; tests/landing-page.mjs; CHANGELOG.html</x:v>
       </x:c>
-      <x:c r="S59" s="14" t="str"/>
+      <x:c r="S59" s="14" t="str">
+        <x:v>3a3c914</x:v>
+      </x:c>
       <x:c r="T59" s="14" t="str">
         <x:v>Run node tests/landing-page.mjs and inspect desktop/mobile rendering.</x:v>
       </x:c>
@@ -4618,7 +4620,7 @@
         <x:v>Rows With Commit Hash</x:v>
       </x:c>
       <x:c r="E9" s="21" t="n">
-        <x:v>8</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">

</xml_diff>